<commit_message>
Map a few existing snippets to APIs
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/outlook.xlsx
+++ b/snippet-extractor-metadata/outlook.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29509"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30004"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF28B44-1C9C-4840-B2EF-A86B2CEA95C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E278CF00-DD2C-4402-B879-80D5F932BEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20250" yWindow="75" windowWidth="36285" windowHeight="20835" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Snippets" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1601" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1606" uniqueCount="345">
   <si>
     <t>Class</t>
   </si>
@@ -1060,6 +1060,9 @@
   </si>
   <si>
     <t>MailboxEnums.TokenStatus</t>
+  </si>
+  <si>
+    <t>SeriesTime</t>
   </si>
 </sst>
 </file>
@@ -1142,10 +1145,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F320" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:F320" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F320">
-    <sortCondition ref="B1:B320"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F321" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:F321" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F321">
+    <sortCondition ref="B1:B321"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{EFF7BB35-6FE7-4943-B8A3-9C5F576D40BA}" name="Package"/>
@@ -1476,7 +1479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F320"/>
+  <dimension ref="A1:F321"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -3674,17 +3677,17 @@
       <c r="A117" t="s">
         <v>226</v>
       </c>
-      <c r="B117" s="2" t="s">
+      <c r="B117" t="s">
         <v>296</v>
       </c>
-      <c r="C117" s="2" t="s">
+      <c r="C117" t="s">
         <v>339</v>
       </c>
-      <c r="D117" s="3"/>
-      <c r="E117" s="2" t="s">
+      <c r="D117" s="1"/>
+      <c r="E117" t="s">
         <v>340</v>
       </c>
-      <c r="F117" s="2" t="s">
+      <c r="F117" t="s">
         <v>341</v>
       </c>
     </row>
@@ -3820,7 +3823,7 @@
         <v>226</v>
       </c>
       <c r="B125" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D125" s="1" t="s">
         <v>288</v>
@@ -3837,7 +3840,7 @@
         <v>226</v>
       </c>
       <c r="B126" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D126" s="1" t="s">
         <v>288</v>
@@ -3913,17 +3916,16 @@
       <c r="A130" t="s">
         <v>226</v>
       </c>
-      <c r="B130" s="2" t="s">
+      <c r="B130" t="s">
         <v>342</v>
       </c>
-      <c r="C130" s="2"/>
-      <c r="D130" s="3" t="s">
+      <c r="D130" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="E130" s="2" t="s">
+      <c r="E130" t="s">
         <v>340</v>
       </c>
-      <c r="F130" s="2" t="s">
+      <c r="F130" t="s">
         <v>341</v>
       </c>
     </row>
@@ -4861,17 +4863,16 @@
       <c r="A181" t="s">
         <v>226</v>
       </c>
-      <c r="B181" s="2" t="s">
+      <c r="B181" t="s">
         <v>343</v>
       </c>
-      <c r="C181" s="2"/>
-      <c r="D181" s="3" t="s">
+      <c r="D181" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="E181" s="2" t="s">
+      <c r="E181" t="s">
         <v>340</v>
       </c>
-      <c r="F181" s="2" t="s">
+      <c r="F181" t="s">
         <v>341</v>
       </c>
     </row>
@@ -7347,20 +7348,18 @@
       <c r="A312" t="s">
         <v>226</v>
       </c>
-      <c r="B312" t="s">
-        <v>198</v>
-      </c>
-      <c r="C312" t="s">
-        <v>202</v>
-      </c>
-      <c r="D312" s="1">
-        <v>1</v>
-      </c>
-      <c r="E312" t="s">
-        <v>272</v>
-      </c>
-      <c r="F312" t="s">
-        <v>203</v>
+      <c r="B312" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C312" s="2"/>
+      <c r="D312" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E312" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F312" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="313" spans="1:6" x14ac:dyDescent="0.25">
@@ -7371,7 +7370,7 @@
         <v>198</v>
       </c>
       <c r="C313" t="s">
-        <v>62</v>
+        <v>202</v>
       </c>
       <c r="D313" s="1">
         <v>1</v>
@@ -7380,7 +7379,7 @@
         <v>272</v>
       </c>
       <c r="F313" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.25">
@@ -7391,7 +7390,7 @@
         <v>198</v>
       </c>
       <c r="C314" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="D314" s="1">
         <v>1</v>
@@ -7400,7 +7399,7 @@
         <v>272</v>
       </c>
       <c r="F314" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="315" spans="1:6" x14ac:dyDescent="0.25">
@@ -7411,7 +7410,7 @@
         <v>198</v>
       </c>
       <c r="C315" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="D315" s="1">
         <v>1</v>
@@ -7420,7 +7419,7 @@
         <v>272</v>
       </c>
       <c r="F315" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.25">
@@ -7431,7 +7430,7 @@
         <v>198</v>
       </c>
       <c r="C316" t="s">
-        <v>133</v>
+        <v>66</v>
       </c>
       <c r="D316" s="1">
         <v>1</v>
@@ -7440,7 +7439,7 @@
         <v>272</v>
       </c>
       <c r="F316" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="317" spans="1:6" x14ac:dyDescent="0.25">
@@ -7448,16 +7447,19 @@
         <v>226</v>
       </c>
       <c r="B317" t="s">
-        <v>311</v>
-      </c>
-      <c r="D317" s="1" t="s">
-        <v>288</v>
+        <v>198</v>
+      </c>
+      <c r="C317" t="s">
+        <v>133</v>
+      </c>
+      <c r="D317" s="1">
+        <v>1</v>
       </c>
       <c r="E317" t="s">
-        <v>103</v>
+        <v>272</v>
       </c>
       <c r="F317" t="s">
-        <v>11</v>
+        <v>199</v>
       </c>
     </row>
     <row r="318" spans="1:6" x14ac:dyDescent="0.25">
@@ -7465,19 +7467,16 @@
         <v>226</v>
       </c>
       <c r="B318" t="s">
-        <v>160</v>
-      </c>
-      <c r="C318" t="s">
-        <v>80</v>
-      </c>
-      <c r="D318" s="1">
-        <v>2</v>
+        <v>311</v>
+      </c>
+      <c r="D318" s="1" t="s">
+        <v>288</v>
       </c>
       <c r="E318" t="s">
-        <v>159</v>
+        <v>103</v>
       </c>
       <c r="F318" t="s">
-        <v>335</v>
+        <v>11</v>
       </c>
     </row>
     <row r="319" spans="1:6" x14ac:dyDescent="0.25">
@@ -7488,16 +7487,16 @@
         <v>160</v>
       </c>
       <c r="C319" t="s">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="D319" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E319" t="s">
         <v>159</v>
       </c>
       <c r="F319" t="s">
-        <v>3</v>
+        <v>335</v>
       </c>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.25">
@@ -7514,9 +7513,29 @@
         <v>1</v>
       </c>
       <c r="E320" t="s">
+        <v>159</v>
+      </c>
+      <c r="F320" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A321" t="s">
+        <v>226</v>
+      </c>
+      <c r="B321" t="s">
+        <v>160</v>
+      </c>
+      <c r="C321" t="s">
+        <v>133</v>
+      </c>
+      <c r="D321" s="1">
+        <v>1</v>
+      </c>
+      <c r="E321" t="s">
         <v>172</v>
       </c>
-      <c r="F320" t="s">
+      <c r="F321" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Map a few existing snippets to APIs (#1085)
</commit_message>
<xml_diff>
--- a/snippet-extractor-metadata/outlook.xlsx
+++ b/snippet-extractor-metadata/outlook.xlsx
@@ -1,11 +1,11 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29509"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30004"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="166925"/>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ABF28B44-1C9C-4840-B2EF-A86B2CEA95C4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E278CF00-DD2C-4402-B879-80D5F932BEC3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20250" yWindow="75" windowWidth="36285" windowHeight="20835" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{CB5595D7-4492-4192-A1C1-2583BA1957AA}"/>
   </bookViews>
   <sheets>
     <sheet name="Snippets" sheetId="2" r:id="rId1"/>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1601" uniqueCount="344">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1606" uniqueCount="345">
   <si>
     <t>Class</t>
   </si>
@@ -1060,6 +1060,9 @@
   </si>
   <si>
     <t>MailboxEnums.TokenStatus</t>
+  </si>
+  <si>
+    <t>SeriesTime</t>
   </si>
 </sst>
 </file>
@@ -1142,10 +1145,10 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F320" totalsRowShown="0" headerRowDxfId="5">
-  <autoFilter ref="A1:F320" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
-  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F320">
-    <sortCondition ref="B1:B320"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{78C585A5-D505-49C6-9CA1-8E6558948317}" name="Snippets" displayName="Snippets" ref="A1:F321" totalsRowShown="0" headerRowDxfId="5">
+  <autoFilter ref="A1:F321" xr:uid="{EAC65D03-FDD2-4352-A5F3-1CDEDE6251B2}"/>
+  <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:F321">
+    <sortCondition ref="B1:B321"/>
   </sortState>
   <tableColumns count="6">
     <tableColumn id="6" xr3:uid="{EFF7BB35-6FE7-4943-B8A3-9C5F576D40BA}" name="Package"/>
@@ -1476,7 +1479,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{809930CD-A227-47DC-AAA4-BB816AEDEB59}">
-  <dimension ref="A1:F320"/>
+  <dimension ref="A1:F321"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10.42578125" bestFit="1" customWidth="1"/>
@@ -3674,17 +3677,17 @@
       <c r="A117" t="s">
         <v>226</v>
       </c>
-      <c r="B117" s="2" t="s">
+      <c r="B117" t="s">
         <v>296</v>
       </c>
-      <c r="C117" s="2" t="s">
+      <c r="C117" t="s">
         <v>339</v>
       </c>
-      <c r="D117" s="3"/>
-      <c r="E117" s="2" t="s">
+      <c r="D117" s="1"/>
+      <c r="E117" t="s">
         <v>340</v>
       </c>
-      <c r="F117" s="2" t="s">
+      <c r="F117" t="s">
         <v>341</v>
       </c>
     </row>
@@ -3820,7 +3823,7 @@
         <v>226</v>
       </c>
       <c r="B125" t="s">
-        <v>332</v>
+        <v>333</v>
       </c>
       <c r="D125" s="1" t="s">
         <v>288</v>
@@ -3837,7 +3840,7 @@
         <v>226</v>
       </c>
       <c r="B126" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D126" s="1" t="s">
         <v>288</v>
@@ -3913,17 +3916,16 @@
       <c r="A130" t="s">
         <v>226</v>
       </c>
-      <c r="B130" s="2" t="s">
+      <c r="B130" t="s">
         <v>342</v>
       </c>
-      <c r="C130" s="2"/>
-      <c r="D130" s="3" t="s">
+      <c r="D130" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="E130" s="2" t="s">
+      <c r="E130" t="s">
         <v>340</v>
       </c>
-      <c r="F130" s="2" t="s">
+      <c r="F130" t="s">
         <v>341</v>
       </c>
     </row>
@@ -4861,17 +4863,16 @@
       <c r="A181" t="s">
         <v>226</v>
       </c>
-      <c r="B181" s="2" t="s">
+      <c r="B181" t="s">
         <v>343</v>
       </c>
-      <c r="C181" s="2"/>
-      <c r="D181" s="3" t="s">
+      <c r="D181" s="1" t="s">
         <v>213</v>
       </c>
-      <c r="E181" s="2" t="s">
+      <c r="E181" t="s">
         <v>340</v>
       </c>
-      <c r="F181" s="2" t="s">
+      <c r="F181" t="s">
         <v>341</v>
       </c>
     </row>
@@ -7347,20 +7348,18 @@
       <c r="A312" t="s">
         <v>226</v>
       </c>
-      <c r="B312" t="s">
-        <v>198</v>
-      </c>
-      <c r="C312" t="s">
-        <v>202</v>
-      </c>
-      <c r="D312" s="1">
-        <v>1</v>
-      </c>
-      <c r="E312" t="s">
-        <v>272</v>
-      </c>
-      <c r="F312" t="s">
-        <v>203</v>
+      <c r="B312" s="2" t="s">
+        <v>344</v>
+      </c>
+      <c r="C312" s="2"/>
+      <c r="D312" s="3" t="s">
+        <v>288</v>
+      </c>
+      <c r="E312" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="F312" s="2" t="s">
+        <v>3</v>
       </c>
     </row>
     <row r="313" spans="1:6" x14ac:dyDescent="0.25">
@@ -7371,7 +7370,7 @@
         <v>198</v>
       </c>
       <c r="C313" t="s">
-        <v>62</v>
+        <v>202</v>
       </c>
       <c r="D313" s="1">
         <v>1</v>
@@ -7380,7 +7379,7 @@
         <v>272</v>
       </c>
       <c r="F313" t="s">
-        <v>197</v>
+        <v>203</v>
       </c>
     </row>
     <row r="314" spans="1:6" x14ac:dyDescent="0.25">
@@ -7391,7 +7390,7 @@
         <v>198</v>
       </c>
       <c r="C314" t="s">
-        <v>80</v>
+        <v>62</v>
       </c>
       <c r="D314" s="1">
         <v>1</v>
@@ -7400,7 +7399,7 @@
         <v>272</v>
       </c>
       <c r="F314" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
     </row>
     <row r="315" spans="1:6" x14ac:dyDescent="0.25">
@@ -7411,7 +7410,7 @@
         <v>198</v>
       </c>
       <c r="C315" t="s">
-        <v>66</v>
+        <v>80</v>
       </c>
       <c r="D315" s="1">
         <v>1</v>
@@ -7420,7 +7419,7 @@
         <v>272</v>
       </c>
       <c r="F315" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
     </row>
     <row r="316" spans="1:6" x14ac:dyDescent="0.25">
@@ -7431,7 +7430,7 @@
         <v>198</v>
       </c>
       <c r="C316" t="s">
-        <v>133</v>
+        <v>66</v>
       </c>
       <c r="D316" s="1">
         <v>1</v>
@@ -7440,7 +7439,7 @@
         <v>272</v>
       </c>
       <c r="F316" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
     </row>
     <row r="317" spans="1:6" x14ac:dyDescent="0.25">
@@ -7448,16 +7447,19 @@
         <v>226</v>
       </c>
       <c r="B317" t="s">
-        <v>311</v>
-      </c>
-      <c r="D317" s="1" t="s">
-        <v>288</v>
+        <v>198</v>
+      </c>
+      <c r="C317" t="s">
+        <v>133</v>
+      </c>
+      <c r="D317" s="1">
+        <v>1</v>
       </c>
       <c r="E317" t="s">
-        <v>103</v>
+        <v>272</v>
       </c>
       <c r="F317" t="s">
-        <v>11</v>
+        <v>199</v>
       </c>
     </row>
     <row r="318" spans="1:6" x14ac:dyDescent="0.25">
@@ -7465,19 +7467,16 @@
         <v>226</v>
       </c>
       <c r="B318" t="s">
-        <v>160</v>
-      </c>
-      <c r="C318" t="s">
-        <v>80</v>
-      </c>
-      <c r="D318" s="1">
-        <v>2</v>
+        <v>311</v>
+      </c>
+      <c r="D318" s="1" t="s">
+        <v>288</v>
       </c>
       <c r="E318" t="s">
-        <v>159</v>
+        <v>103</v>
       </c>
       <c r="F318" t="s">
-        <v>335</v>
+        <v>11</v>
       </c>
     </row>
     <row r="319" spans="1:6" x14ac:dyDescent="0.25">
@@ -7488,16 +7487,16 @@
         <v>160</v>
       </c>
       <c r="C319" t="s">
-        <v>133</v>
+        <v>80</v>
       </c>
       <c r="D319" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E319" t="s">
         <v>159</v>
       </c>
       <c r="F319" t="s">
-        <v>3</v>
+        <v>335</v>
       </c>
     </row>
     <row r="320" spans="1:6" x14ac:dyDescent="0.25">
@@ -7514,9 +7513,29 @@
         <v>1</v>
       </c>
       <c r="E320" t="s">
+        <v>159</v>
+      </c>
+      <c r="F320" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="321" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="A321" t="s">
+        <v>226</v>
+      </c>
+      <c r="B321" t="s">
+        <v>160</v>
+      </c>
+      <c r="C321" t="s">
+        <v>133</v>
+      </c>
+      <c r="D321" s="1">
+        <v>1</v>
+      </c>
+      <c r="E321" t="s">
         <v>172</v>
       </c>
-      <c r="F320" t="s">
+      <c r="F321" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>